<commit_message>
Test case for LMS
</commit_message>
<xml_diff>
--- a/TEST CASE CAPGEMINI TRAINING.xlsx
+++ b/TEST CASE CAPGEMINI TRAINING.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARYAN\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6aedb703216c14ed/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937BDF8C-D4E1-4A4C-8D4D-E880C43C15EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{937BDF8C-D4E1-4A4C-8D4D-E880C43C15EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C3FB77D-86A7-49AC-BD18-A55E7DD17752}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="643">
   <si>
     <t>APPLICATION NAME</t>
   </si>
@@ -1328,12 +1329,699 @@
   <si>
     <t>LMS_UM_076</t>
   </si>
+  <si>
+    <t>1.2 UPDATE USER</t>
+  </si>
+  <si>
+    <t>USER SHOULD BE LOGGED IN AND NAVIGATED TO UPDATE USER PAGE</t>
+  </si>
+  <si>
+    <t>VERIFY THE FUNCTIONALITY OF UPDATE USER MODULE</t>
+  </si>
+  <si>
+    <t>TEST TYPE</t>
+  </si>
+  <si>
+    <t>USER_ID_VALID</t>
+  </si>
+  <si>
+    <t>FUNCTIONAL</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM ACCEPTS VALID NUMERIC USER ID</t>
+  </si>
+  <si>
+    <t>1. OPEN APP 2. NAVIGATE TO UPDATE USER 3. ENTER USER ID</t>
+  </si>
+  <si>
+    <t>USER ID ACCEPTED</t>
+  </si>
+  <si>
+    <t>USER_ID_FETCH</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM DISPLAYS USER DETAILS FOR VALID ID</t>
+  </si>
+  <si>
+    <t>1. OPEN APP 2. ENTER VALID USER ID 3. CLICK SEARCH</t>
+  </si>
+  <si>
+    <t>EXISTING ID</t>
+  </si>
+  <si>
+    <t>USER DETAILS DISPLAYED</t>
+  </si>
+  <si>
+    <t>USER_ID_ALPHA</t>
+  </si>
+  <si>
+    <t>NEGATIVE</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM REJECTS USER ID WITH ALPHABETS</t>
+  </si>
+  <si>
+    <t>1. ENTER USER ID</t>
+  </si>
+  <si>
+    <t>ABC123</t>
+  </si>
+  <si>
+    <t>ERROR MESSAGE DISPLAYED</t>
+  </si>
+  <si>
+    <t>USER_ID_SPECIAL</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM REJECTS USER ID WITH SPECIAL CHARACTERS</t>
+  </si>
+  <si>
+    <t>USER_ID_MAX</t>
+  </si>
+  <si>
+    <t>BOUNDARY</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM ACCEPTS 10 DIGIT USER ID</t>
+  </si>
+  <si>
+    <t>ACCEPTED</t>
+  </si>
+  <si>
+    <t>USER_ID_ABOVE_MAX</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM REJECTS USER ID &gt;10 DIGITS</t>
+  </si>
+  <si>
+    <t>ERROR MESSAGE</t>
+  </si>
+  <si>
+    <t>USER_ID_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM SHOWS MESSAGE FOR INVALID USER</t>
+  </si>
+  <si>
+    <t>1. ENTER USER ID 2. SEARCH</t>
+  </si>
+  <si>
+    <t>"USER NOT FOUND"</t>
+  </si>
+  <si>
+    <t>USER_ID_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY SYSTEM REJECTS BLANK USER ID</t>
+  </si>
+  <si>
+    <t>1. LEAVE FIELD EMPTY 2. CLICK SEARCH</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>FN_VALID</t>
+  </si>
+  <si>
+    <t>VERIFY ACCEPTS VALID FIRST NAME</t>
+  </si>
+  <si>
+    <t>1. ENTER FIRST NAME</t>
+  </si>
+  <si>
+    <t>FN_NUMERIC</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS NUMERIC INPUT</t>
+  </si>
+  <si>
+    <t>ERROR</t>
+  </si>
+  <si>
+    <t>FN_SPECIAL</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS SPECIAL CHARACTERS</t>
+  </si>
+  <si>
+    <t>FN_MAX</t>
+  </si>
+  <si>
+    <t>VERIFY ACCEPTS 25 CHAR</t>
+  </si>
+  <si>
+    <t>1. ENTER VALUE</t>
+  </si>
+  <si>
+    <t>25 CHAR STRING</t>
+  </si>
+  <si>
+    <t>FN_ABOVE_MAX</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS &gt;25 CHAR</t>
+  </si>
+  <si>
+    <t>26 CHAR STRING</t>
+  </si>
+  <si>
+    <t>FN_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS BLANK</t>
+  </si>
+  <si>
+    <t>1. LEAVE EMPTY</t>
+  </si>
+  <si>
+    <t>LN_VALID</t>
+  </si>
+  <si>
+    <t>VERIFY ACCEPTS VALID LAST NAME</t>
+  </si>
+  <si>
+    <t>ENTER LAST NAME</t>
+  </si>
+  <si>
+    <t>LN_NUMERIC</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS NUMBERS</t>
+  </si>
+  <si>
+    <t>ENTER VALUE</t>
+  </si>
+  <si>
+    <t>LN_SPECIAL</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS SPECIAL CHAR</t>
+  </si>
+  <si>
+    <t>LN_MAX</t>
+  </si>
+  <si>
+    <t>VERIFY ACCEPTS 30 CHAR</t>
+  </si>
+  <si>
+    <t>30 CHAR</t>
+  </si>
+  <si>
+    <t>LN_ABOVE_MAX</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS &gt;30 CHAR</t>
+  </si>
+  <si>
+    <t>31 CHAR</t>
+  </si>
+  <si>
+    <t>LN_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY BLANK NOT ALLOWED</t>
+  </si>
+  <si>
+    <t>LEAVE EMPTY</t>
+  </si>
+  <si>
+    <t>EMAIL_VALID</t>
+  </si>
+  <si>
+    <t>VERIFY ACCEPTS VALID EMAIL</t>
+  </si>
+  <si>
+    <t>ENTER EMAIL</t>
+  </si>
+  <si>
+    <t>EMAIL_INVALID</t>
+  </si>
+  <si>
+    <t>VERIFY INVALID FORMAT</t>
+  </si>
+  <si>
+    <t>testgmail.com</t>
+  </si>
+  <si>
+    <t>EMAIL_DUPLICATE</t>
+  </si>
+  <si>
+    <t>VERIFY DUPLICATE EMAIL</t>
+  </si>
+  <si>
+    <t>existing@gmail.com</t>
+  </si>
+  <si>
+    <t>EMAIL_UNIQUE</t>
+  </si>
+  <si>
+    <t>VERIFY UNIQUE EMAIL ACCEPTED</t>
+  </si>
+  <si>
+    <t>new@gmail.com</t>
+  </si>
+  <si>
+    <t>EMAIL_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY BLANK EMAIL</t>
+  </si>
+  <si>
+    <t>PHONE_VALID</t>
+  </si>
+  <si>
+    <t>VERIFY VALID PHONE NUMBER</t>
+  </si>
+  <si>
+    <t>ENTER PHONE</t>
+  </si>
+  <si>
+    <t>PHONE_ALPHA</t>
+  </si>
+  <si>
+    <t>VERIFY REJECTS ALPHABETS</t>
+  </si>
+  <si>
+    <t>PHONE_SPECIAL</t>
+  </si>
+  <si>
+    <t>98@#</t>
+  </si>
+  <si>
+    <t>PHONE_SHORT</t>
+  </si>
+  <si>
+    <t>VERIFY &lt;10 DIGITS</t>
+  </si>
+  <si>
+    <t>PHONE_LONG</t>
+  </si>
+  <si>
+    <t>VERIFY &gt;10 DIGITS</t>
+  </si>
+  <si>
+    <t>PHONE_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY BLANK PHONE</t>
+  </si>
+  <si>
+    <t>ROLE_ADMIN</t>
+  </si>
+  <si>
+    <t>VERIFY ADMIN SELECTED</t>
+  </si>
+  <si>
+    <t>SELECT ROLE</t>
+  </si>
+  <si>
+    <t>ADMIN</t>
+  </si>
+  <si>
+    <t>ROLE_LIBRARIAN</t>
+  </si>
+  <si>
+    <t>VERIFY LIBRARIAN SELECTED</t>
+  </si>
+  <si>
+    <t>LIBRARIAN</t>
+  </si>
+  <si>
+    <t>ROLE_MEMBER</t>
+  </si>
+  <si>
+    <t>VERIFY MEMBER SELECTED</t>
+  </si>
+  <si>
+    <t>MEMBER</t>
+  </si>
+  <si>
+    <t>ROLE_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY NO SELECTION</t>
+  </si>
+  <si>
+    <t>DO NOT SELECT</t>
+  </si>
+  <si>
+    <t>STATUS_ACTIVE</t>
+  </si>
+  <si>
+    <t>VERIFY ACTIVE SELECTED</t>
+  </si>
+  <si>
+    <t>SELECT STATUS</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>SELECTED</t>
+  </si>
+  <si>
+    <t>STATUS_INACTIVE</t>
+  </si>
+  <si>
+    <t>VERIFY INACTIVE SELECTED</t>
+  </si>
+  <si>
+    <t>INACTIVE</t>
+  </si>
+  <si>
+    <t>STATUS_MULTI</t>
+  </si>
+  <si>
+    <t>VERIFY ONLY ONE SELECTION</t>
+  </si>
+  <si>
+    <t>TRY SELECT BOTH</t>
+  </si>
+  <si>
+    <t>BOTH</t>
+  </si>
+  <si>
+    <t>NOT ALLOWED</t>
+  </si>
+  <si>
+    <t>STATUS_BLANK</t>
+  </si>
+  <si>
+    <t>VERIFY NO STATUS</t>
+  </si>
+  <si>
+    <t>UPDATE_VALID</t>
+  </si>
+  <si>
+    <t>INTEGRATION</t>
+  </si>
+  <si>
+    <t>VERIFY UPDATE WITH VALID DATA</t>
+  </si>
+  <si>
+    <t>1. ENTER ALL VALID DATA 2. CLICK UPDATE</t>
+  </si>
+  <si>
+    <t>VALID DATA</t>
+  </si>
+  <si>
+    <t>USER UPDATED</t>
+  </si>
+  <si>
+    <t>UPDATE_INVALID</t>
+  </si>
+  <si>
+    <t>VERIFY UPDATE WITH INVALID DATA</t>
+  </si>
+  <si>
+    <t>ENTER INVALID DATA</t>
+  </si>
+  <si>
+    <t>INVALID DATA</t>
+  </si>
+  <si>
+    <t>UPDATE_EMPTY</t>
+  </si>
+  <si>
+    <t>VERIFY EMPTY FIELDS</t>
+  </si>
+  <si>
+    <t>LEAVE FIELDS EMPTY</t>
+  </si>
+  <si>
+    <t>UPDATE_DUP_EMAIL</t>
+  </si>
+  <si>
+    <t>ENTER DUP EMAIL</t>
+  </si>
+  <si>
+    <t>UPDATE_NO_CHANGE</t>
+  </si>
+  <si>
+    <t>VERIFY NO CHANGE CASE</t>
+  </si>
+  <si>
+    <t>CLICK UPDATE WITHOUT CHANGE</t>
+  </si>
+  <si>
+    <t>SAME DATA</t>
+  </si>
+  <si>
+    <t>"NO CHANGES DETECTED"</t>
+  </si>
+  <si>
+    <t>UPDATE_SUCCESS</t>
+  </si>
+  <si>
+    <t>VERIFY SUCCESS MESSAGE</t>
+  </si>
+  <si>
+    <t>CLICK UPDATE</t>
+  </si>
+  <si>
+    <t>SUCCESS MESSAGE</t>
+  </si>
+  <si>
+    <t>UPDATE_VALIDATE</t>
+  </si>
+  <si>
+    <t>VERIFY FIELD VALIDATION</t>
+  </si>
+  <si>
+    <t>VALIDATION ERRORS</t>
+  </si>
+  <si>
+    <t>CANCEL_CLEAR</t>
+  </si>
+  <si>
+    <t>VERIFY FIELDS RESET</t>
+  </si>
+  <si>
+    <t>MODIFY DATA → CLICK CANCEL</t>
+  </si>
+  <si>
+    <t>MODIFIED DATA</t>
+  </si>
+  <si>
+    <t>FIELDS CLEARED</t>
+  </si>
+  <si>
+    <t>CANCEL_REDIRECT</t>
+  </si>
+  <si>
+    <t>VERIFY REDIRECTION</t>
+  </si>
+  <si>
+    <t>CLICK CANCEL</t>
+  </si>
+  <si>
+    <t>REDIRECT TO LIST</t>
+  </si>
+  <si>
+    <t>CANCEL_DISCARD</t>
+  </si>
+  <si>
+    <t>VERIFY NO SAVE</t>
+  </si>
+  <si>
+    <t>MODIFY DATA → CANCEL</t>
+  </si>
+  <si>
+    <t>DATA NOT SAVED</t>
+  </si>
+  <si>
+    <t>CANCEL_NO_CHANGE</t>
+  </si>
+  <si>
+    <t>VERIFY CANCEL WITHOUT CHANGE</t>
+  </si>
+  <si>
+    <t>REDIRECT</t>
+  </si>
+  <si>
+    <t>123@$</t>
+  </si>
+  <si>
+    <t>Aryan</t>
+  </si>
+  <si>
+    <t>Ary123</t>
+  </si>
+  <si>
+    <t>Ary@#</t>
+  </si>
+  <si>
+    <t>Sharma</t>
+  </si>
+  <si>
+    <t>Sharma@</t>
+  </si>
+  <si>
+    <t>sharma123</t>
+  </si>
+  <si>
+    <t>aryan@gmail.com</t>
+  </si>
+  <si>
+    <t>USER LOGIN</t>
+  </si>
+  <si>
+    <t>LMS_UL_001</t>
+  </si>
+  <si>
+    <t>LMS_UL_002</t>
+  </si>
+  <si>
+    <t>LMS_UL_003</t>
+  </si>
+  <si>
+    <t>LMS_UL_004</t>
+  </si>
+  <si>
+    <t>LMS_UL_005</t>
+  </si>
+  <si>
+    <t>LMS_UL_006</t>
+  </si>
+  <si>
+    <t>LMS_UL_007</t>
+  </si>
+  <si>
+    <t>LMS_UL_008</t>
+  </si>
+  <si>
+    <t>LMS_UL_009</t>
+  </si>
+  <si>
+    <t>LMS_UL_010</t>
+  </si>
+  <si>
+    <t>LMS_UL_011</t>
+  </si>
+  <si>
+    <t>LMS_UL_012</t>
+  </si>
+  <si>
+    <t>LMS_UL_013</t>
+  </si>
+  <si>
+    <t>LMS_UL_014</t>
+  </si>
+  <si>
+    <t>LMS_UL_015</t>
+  </si>
+  <si>
+    <t>LMS_UL_016</t>
+  </si>
+  <si>
+    <t>LMS_UL_017</t>
+  </si>
+  <si>
+    <t>LMS_UL_018</t>
+  </si>
+  <si>
+    <t>LMS_UL_019</t>
+  </si>
+  <si>
+    <t>LMS_UL_020</t>
+  </si>
+  <si>
+    <t>LMS_UL_021</t>
+  </si>
+  <si>
+    <t>LMS_UL_022</t>
+  </si>
+  <si>
+    <t>LMS_UL_023</t>
+  </si>
+  <si>
+    <t>LMS_UL_024</t>
+  </si>
+  <si>
+    <t>LMS_UL_025</t>
+  </si>
+  <si>
+    <t>LMS_UL_026</t>
+  </si>
+  <si>
+    <t>LMS_UL_027</t>
+  </si>
+  <si>
+    <t>LMS_UL_028</t>
+  </si>
+  <si>
+    <t>LMS_UL_029</t>
+  </si>
+  <si>
+    <t>LMS_UL_030</t>
+  </si>
+  <si>
+    <t>LMS_UL_031</t>
+  </si>
+  <si>
+    <t>LMS_UL_032</t>
+  </si>
+  <si>
+    <t>LMS_UL_033</t>
+  </si>
+  <si>
+    <t>LMS_UL_034</t>
+  </si>
+  <si>
+    <t>LMS_UL_035</t>
+  </si>
+  <si>
+    <t>LMS_UL_036</t>
+  </si>
+  <si>
+    <t>LMS_UL_037</t>
+  </si>
+  <si>
+    <t>LMS_UL_038</t>
+  </si>
+  <si>
+    <t>LMS_UL_039</t>
+  </si>
+  <si>
+    <t>LMS_UL_040</t>
+  </si>
+  <si>
+    <t>LMS_UL_041</t>
+  </si>
+  <si>
+    <t>LMS_UL_042</t>
+  </si>
+  <si>
+    <t>LMS_UL_043</t>
+  </si>
+  <si>
+    <t>LMS_UL_044</t>
+  </si>
+  <si>
+    <t>LMS_UL_045</t>
+  </si>
+  <si>
+    <t>LMS_UL_046</t>
+  </si>
+  <si>
+    <t>LMS_UL_047</t>
+  </si>
+  <si>
+    <t>LMS_UL_048</t>
+  </si>
+  <si>
+    <t>LMS_UL_049</t>
+  </si>
+  <si>
+    <t>LMS_UL_050</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1374,6 +2062,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1411,7 +2107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1439,13 +2135,29 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2230,87 +2942,87 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C25" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D25" s="12" t="s">
+      <c r="C25" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" s="13" t="s">
         <v>107</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="G25" s="13" t="s">
+      <c r="G25" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
       <c r="E26" s="9"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="12"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
       <c r="E27" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F27" s="12"/>
-      <c r="G27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="12"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="9"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="12"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
       <c r="E29" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="F29" s="12"/>
-      <c r="G29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="12"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
       <c r="E30" s="9"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="12"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
       <c r="E31" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="12"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
@@ -2681,16 +3393,16 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="13" t="s">
         <v>245</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="C48" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D48" s="12" t="s">
+      <c r="C48" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D48" s="13" t="s">
         <v>186</v>
       </c>
       <c r="E48" s="7" t="s">
@@ -2699,134 +3411,134 @@
       <c r="F48" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="G48" s="13" t="s">
+      <c r="G48" s="12" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="12"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
+      <c r="A49" s="13"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
-      <c r="G49" s="13"/>
+      <c r="G49" s="12"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="12"/>
-      <c r="B50" s="12"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="12"/>
+      <c r="A50" s="13"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
       <c r="E50" s="7" t="s">
         <v>109</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="G50" s="13"/>
+      <c r="G50" s="12"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A51" s="12"/>
-      <c r="B51" s="12"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="12"/>
+      <c r="A51" s="13"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
-      <c r="G51" s="13"/>
+      <c r="G51" s="12"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="12"/>
-      <c r="B52" s="12"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
+      <c r="A52" s="13"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="13"/>
       <c r="E52" s="7" t="s">
         <v>110</v>
       </c>
       <c r="F52" s="9"/>
-      <c r="G52" s="13"/>
+      <c r="G52" s="12"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" s="12"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
+      <c r="A53" s="13"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
       <c r="E53" s="9"/>
       <c r="F53" s="9"/>
-      <c r="G53" s="13"/>
+      <c r="G53" s="12"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A54" s="12"/>
-      <c r="B54" s="12"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
+      <c r="A54" s="13"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
       <c r="E54" s="7" t="s">
         <v>187</v>
       </c>
       <c r="F54" s="9"/>
-      <c r="G54" s="13"/>
+      <c r="G54" s="12"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" s="12"/>
-      <c r="B55" s="12"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="12"/>
+      <c r="A55" s="13"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
       <c r="E55" s="9"/>
       <c r="F55" s="9"/>
-      <c r="G55" s="13"/>
+      <c r="G55" s="12"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A56" s="12"/>
-      <c r="B56" s="12"/>
-      <c r="C56" s="12"/>
-      <c r="D56" s="12"/>
+      <c r="A56" s="13"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="13"/>
+      <c r="D56" s="13"/>
       <c r="E56" s="7" t="s">
         <v>188</v>
       </c>
       <c r="F56" s="9"/>
-      <c r="G56" s="13"/>
+      <c r="G56" s="12"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="C57" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D57" s="12" t="s">
+      <c r="C57" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D57" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="E57" s="12" t="s">
+      <c r="E57" s="13" t="s">
         <v>195</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="G57" s="13" t="s">
+      <c r="G57" s="12" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" s="12"/>
-      <c r="B58" s="12"/>
-      <c r="C58" s="12"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="12"/>
+      <c r="A58" s="13"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="13"/>
       <c r="F58" s="9"/>
-      <c r="G58" s="13"/>
+      <c r="G58" s="12"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A59" s="12"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
+      <c r="A59" s="13"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="13"/>
+      <c r="D59" s="13"/>
+      <c r="E59" s="13"/>
       <c r="F59" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="G59" s="13"/>
+      <c r="G59" s="12"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="7" t="s">
@@ -2852,87 +3564,87 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D61" s="12" t="s">
+      <c r="C61" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D61" s="13" t="s">
         <v>205</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="F61" s="12" t="s">
+      <c r="F61" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="G61" s="13" t="s">
+      <c r="G61" s="12" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62" s="12"/>
-      <c r="B62" s="12"/>
-      <c r="C62" s="12"/>
-      <c r="D62" s="12"/>
+      <c r="A62" s="13"/>
+      <c r="B62" s="13"/>
+      <c r="C62" s="13"/>
+      <c r="D62" s="13"/>
       <c r="E62" s="9"/>
-      <c r="F62" s="12"/>
-      <c r="G62" s="13"/>
+      <c r="F62" s="13"/>
+      <c r="G62" s="12"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A63" s="12"/>
-      <c r="B63" s="12"/>
-      <c r="C63" s="12"/>
-      <c r="D63" s="12"/>
+      <c r="A63" s="13"/>
+      <c r="B63" s="13"/>
+      <c r="C63" s="13"/>
+      <c r="D63" s="13"/>
       <c r="E63" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F63" s="12"/>
-      <c r="G63" s="13"/>
+      <c r="F63" s="13"/>
+      <c r="G63" s="12"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A64" s="12"/>
-      <c r="B64" s="12"/>
-      <c r="C64" s="12"/>
-      <c r="D64" s="12"/>
+      <c r="A64" s="13"/>
+      <c r="B64" s="13"/>
+      <c r="C64" s="13"/>
+      <c r="D64" s="13"/>
       <c r="E64" s="9"/>
-      <c r="F64" s="12"/>
-      <c r="G64" s="13"/>
+      <c r="F64" s="13"/>
+      <c r="G64" s="12"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" s="12"/>
-      <c r="B65" s="12"/>
-      <c r="C65" s="12"/>
-      <c r="D65" s="12"/>
+      <c r="A65" s="13"/>
+      <c r="B65" s="13"/>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
       <c r="E65" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="F65" s="12"/>
-      <c r="G65" s="13"/>
+      <c r="F65" s="13"/>
+      <c r="G65" s="12"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="12"/>
-      <c r="B66" s="12"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="12"/>
+      <c r="A66" s="13"/>
+      <c r="B66" s="13"/>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
       <c r="E66" s="9"/>
-      <c r="F66" s="12"/>
-      <c r="G66" s="13"/>
+      <c r="F66" s="13"/>
+      <c r="G66" s="12"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67" s="12"/>
-      <c r="B67" s="12"/>
-      <c r="C67" s="12"/>
-      <c r="D67" s="12"/>
+      <c r="A67" s="13"/>
+      <c r="B67" s="13"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="13"/>
       <c r="E67" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="F67" s="12"/>
-      <c r="G67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="12"/>
     </row>
     <row r="68" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A68" s="7" t="s">
@@ -3027,16 +3739,16 @@
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="13" t="s">
         <v>283</v>
       </c>
-      <c r="B72" s="12" t="s">
+      <c r="B72" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="C72" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D72" s="12" t="s">
+      <c r="C72" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D72" s="13" t="s">
         <v>232</v>
       </c>
       <c r="E72" s="7" t="s">
@@ -3045,69 +3757,69 @@
       <c r="F72" s="14">
         <v>34926</v>
       </c>
-      <c r="G72" s="13" t="s">
+      <c r="G72" s="12" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A73" s="12"/>
-      <c r="B73" s="12"/>
-      <c r="C73" s="12"/>
-      <c r="D73" s="12"/>
+      <c r="A73" s="13"/>
+      <c r="B73" s="13"/>
+      <c r="C73" s="13"/>
+      <c r="D73" s="13"/>
       <c r="E73" s="9"/>
       <c r="F73" s="14"/>
-      <c r="G73" s="13"/>
+      <c r="G73" s="12"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A74" s="12"/>
-      <c r="B74" s="12"/>
-      <c r="C74" s="12"/>
-      <c r="D74" s="12"/>
+      <c r="A74" s="13"/>
+      <c r="B74" s="13"/>
+      <c r="C74" s="13"/>
+      <c r="D74" s="13"/>
       <c r="E74" s="7" t="s">
         <v>109</v>
       </c>
       <c r="F74" s="14"/>
-      <c r="G74" s="13"/>
+      <c r="G74" s="12"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A75" s="12"/>
-      <c r="B75" s="12"/>
-      <c r="C75" s="12"/>
-      <c r="D75" s="12"/>
+      <c r="A75" s="13"/>
+      <c r="B75" s="13"/>
+      <c r="C75" s="13"/>
+      <c r="D75" s="13"/>
       <c r="E75" s="9"/>
       <c r="F75" s="14"/>
-      <c r="G75" s="13"/>
+      <c r="G75" s="12"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A76" s="12"/>
-      <c r="B76" s="12"/>
-      <c r="C76" s="12"/>
-      <c r="D76" s="12"/>
+      <c r="A76" s="13"/>
+      <c r="B76" s="13"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="13"/>
       <c r="E76" s="7" t="s">
         <v>110</v>
       </c>
       <c r="F76" s="14"/>
-      <c r="G76" s="13"/>
+      <c r="G76" s="12"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A77" s="12"/>
-      <c r="B77" s="12"/>
-      <c r="C77" s="12"/>
-      <c r="D77" s="12"/>
+      <c r="A77" s="13"/>
+      <c r="B77" s="13"/>
+      <c r="C77" s="13"/>
+      <c r="D77" s="13"/>
       <c r="E77" s="9"/>
       <c r="F77" s="14"/>
-      <c r="G77" s="13"/>
+      <c r="G77" s="12"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" s="12"/>
-      <c r="B78" s="12"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="12"/>
+      <c r="A78" s="13"/>
+      <c r="B78" s="13"/>
+      <c r="C78" s="13"/>
+      <c r="D78" s="13"/>
       <c r="E78" s="7" t="s">
         <v>233</v>
       </c>
       <c r="F78" s="14"/>
-      <c r="G78" s="13"/>
+      <c r="G78" s="12"/>
     </row>
     <row r="79" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A79" s="7" t="s">
@@ -3133,90 +3845,90 @@
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A80" s="12" t="s">
+      <c r="A80" s="13" t="s">
         <v>293</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="C80" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D80" s="12" t="s">
+      <c r="C80" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D80" s="13" t="s">
         <v>241</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="F80" s="12" t="s">
+      <c r="F80" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="G80" s="13" t="s">
+      <c r="G80" s="12" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A81" s="12"/>
-      <c r="B81" s="12"/>
-      <c r="C81" s="12"/>
-      <c r="D81" s="12"/>
+      <c r="A81" s="13"/>
+      <c r="B81" s="13"/>
+      <c r="C81" s="13"/>
+      <c r="D81" s="13"/>
       <c r="E81" s="9"/>
-      <c r="F81" s="12"/>
-      <c r="G81" s="13"/>
+      <c r="F81" s="13"/>
+      <c r="G81" s="12"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A82" s="12"/>
-      <c r="B82" s="12"/>
-      <c r="C82" s="12"/>
-      <c r="D82" s="12"/>
+      <c r="A82" s="13"/>
+      <c r="B82" s="13"/>
+      <c r="C82" s="13"/>
+      <c r="D82" s="13"/>
       <c r="E82" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="F82" s="12"/>
-      <c r="G82" s="13"/>
+      <c r="F82" s="13"/>
+      <c r="G82" s="12"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A83" s="12" t="s">
+      <c r="A83" s="13" t="s">
         <v>297</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="C83" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D83" s="12" t="s">
+      <c r="C83" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D83" s="13" t="s">
         <v>247</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="F83" s="12" t="s">
+      <c r="F83" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="G83" s="13" t="s">
+      <c r="G83" s="12" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A84" s="12"/>
-      <c r="B84" s="12"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
+      <c r="A84" s="13"/>
+      <c r="B84" s="13"/>
+      <c r="C84" s="13"/>
+      <c r="D84" s="13"/>
       <c r="E84" s="9"/>
-      <c r="F84" s="12"/>
-      <c r="G84" s="13"/>
+      <c r="F84" s="13"/>
+      <c r="G84" s="12"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A85" s="12"/>
-      <c r="B85" s="12"/>
-      <c r="C85" s="12"/>
-      <c r="D85" s="12"/>
+      <c r="A85" s="13"/>
+      <c r="B85" s="13"/>
+      <c r="C85" s="13"/>
+      <c r="D85" s="13"/>
       <c r="E85" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="F85" s="12"/>
-      <c r="G85" s="13"/>
+      <c r="F85" s="13"/>
+      <c r="G85" s="12"/>
     </row>
     <row r="86" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A86" s="7" t="s">
@@ -3633,87 +4345,87 @@
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A104" s="12" t="s">
+      <c r="A104" s="13" t="s">
         <v>386</v>
       </c>
-      <c r="B104" s="12" t="s">
+      <c r="B104" s="13" t="s">
         <v>335</v>
       </c>
-      <c r="C104" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D104" s="12" t="s">
+      <c r="C104" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D104" s="13" t="s">
         <v>336</v>
       </c>
       <c r="E104" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="F104" s="12" t="s">
+      <c r="F104" s="13" t="s">
         <v>401</v>
       </c>
-      <c r="G104" s="13" t="s">
+      <c r="G104" s="12" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A105" s="12"/>
-      <c r="B105" s="12"/>
-      <c r="C105" s="12"/>
-      <c r="D105" s="12"/>
+      <c r="A105" s="13"/>
+      <c r="B105" s="13"/>
+      <c r="C105" s="13"/>
+      <c r="D105" s="13"/>
       <c r="E105" s="9"/>
-      <c r="F105" s="12"/>
-      <c r="G105" s="13"/>
+      <c r="F105" s="13"/>
+      <c r="G105" s="12"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A106" s="12"/>
-      <c r="B106" s="12"/>
-      <c r="C106" s="12"/>
-      <c r="D106" s="12"/>
+      <c r="A106" s="13"/>
+      <c r="B106" s="13"/>
+      <c r="C106" s="13"/>
+      <c r="D106" s="13"/>
       <c r="E106" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F106" s="12"/>
-      <c r="G106" s="13"/>
+      <c r="F106" s="13"/>
+      <c r="G106" s="12"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A107" s="12"/>
-      <c r="B107" s="12"/>
-      <c r="C107" s="12"/>
-      <c r="D107" s="12"/>
+      <c r="A107" s="13"/>
+      <c r="B107" s="13"/>
+      <c r="C107" s="13"/>
+      <c r="D107" s="13"/>
       <c r="E107" s="9"/>
-      <c r="F107" s="12"/>
-      <c r="G107" s="13"/>
+      <c r="F107" s="13"/>
+      <c r="G107" s="12"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A108" s="12"/>
-      <c r="B108" s="12"/>
-      <c r="C108" s="12"/>
-      <c r="D108" s="12"/>
+      <c r="A108" s="13"/>
+      <c r="B108" s="13"/>
+      <c r="C108" s="13"/>
+      <c r="D108" s="13"/>
       <c r="E108" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="F108" s="12"/>
-      <c r="G108" s="13"/>
+      <c r="F108" s="13"/>
+      <c r="G108" s="12"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A109" s="12"/>
-      <c r="B109" s="12"/>
-      <c r="C109" s="12"/>
-      <c r="D109" s="12"/>
+      <c r="A109" s="13"/>
+      <c r="B109" s="13"/>
+      <c r="C109" s="13"/>
+      <c r="D109" s="13"/>
       <c r="E109" s="9"/>
-      <c r="F109" s="12"/>
-      <c r="G109" s="13"/>
+      <c r="F109" s="13"/>
+      <c r="G109" s="12"/>
     </row>
     <row r="110" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A110" s="12"/>
-      <c r="B110" s="12"/>
-      <c r="C110" s="12"/>
-      <c r="D110" s="12"/>
+      <c r="A110" s="13"/>
+      <c r="B110" s="13"/>
+      <c r="C110" s="13"/>
+      <c r="D110" s="13"/>
       <c r="E110" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="F110" s="12"/>
-      <c r="G110" s="13"/>
+      <c r="F110" s="13"/>
+      <c r="G110" s="12"/>
     </row>
     <row r="111" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A111" s="7" t="s">
@@ -3808,133 +4520,133 @@
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A115" s="12" t="s">
+      <c r="A115" s="13" t="s">
         <v>406</v>
       </c>
-      <c r="B115" s="12" t="s">
+      <c r="B115" s="13" t="s">
         <v>352</v>
       </c>
-      <c r="C115" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D115" s="12" t="s">
+      <c r="C115" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D115" s="13" t="s">
         <v>353</v>
       </c>
       <c r="E115" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="F115" s="12" t="s">
+      <c r="F115" s="13" t="s">
         <v>355</v>
       </c>
-      <c r="G115" s="13" t="s">
+      <c r="G115" s="12" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A116" s="12"/>
-      <c r="B116" s="12"/>
-      <c r="C116" s="12"/>
-      <c r="D116" s="12"/>
+      <c r="A116" s="13"/>
+      <c r="B116" s="13"/>
+      <c r="C116" s="13"/>
+      <c r="D116" s="13"/>
       <c r="E116" s="9"/>
-      <c r="F116" s="12"/>
-      <c r="G116" s="13"/>
+      <c r="F116" s="13"/>
+      <c r="G116" s="12"/>
     </row>
     <row r="117" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A117" s="12"/>
-      <c r="B117" s="12"/>
-      <c r="C117" s="12"/>
-      <c r="D117" s="12"/>
+      <c r="A117" s="13"/>
+      <c r="B117" s="13"/>
+      <c r="C117" s="13"/>
+      <c r="D117" s="13"/>
       <c r="E117" s="7" t="s">
         <v>354</v>
       </c>
-      <c r="F117" s="12"/>
-      <c r="G117" s="13"/>
+      <c r="F117" s="13"/>
+      <c r="G117" s="12"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A118" s="12" t="s">
+      <c r="A118" s="13" t="s">
         <v>407</v>
       </c>
-      <c r="B118" s="12" t="s">
+      <c r="B118" s="13" t="s">
         <v>358</v>
       </c>
-      <c r="C118" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D118" s="12" t="s">
+      <c r="C118" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D118" s="13" t="s">
         <v>359</v>
       </c>
       <c r="E118" s="7" t="s">
         <v>360</v>
       </c>
-      <c r="F118" s="12" t="s">
+      <c r="F118" s="13" t="s">
         <v>362</v>
       </c>
-      <c r="G118" s="13" t="s">
+      <c r="G118" s="12" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A119" s="12"/>
-      <c r="B119" s="12"/>
-      <c r="C119" s="12"/>
-      <c r="D119" s="12"/>
+      <c r="A119" s="13"/>
+      <c r="B119" s="13"/>
+      <c r="C119" s="13"/>
+      <c r="D119" s="13"/>
       <c r="E119" s="9"/>
-      <c r="F119" s="12"/>
-      <c r="G119" s="13"/>
+      <c r="F119" s="13"/>
+      <c r="G119" s="12"/>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A120" s="12"/>
-      <c r="B120" s="12"/>
-      <c r="C120" s="12"/>
-      <c r="D120" s="12"/>
+      <c r="A120" s="13"/>
+      <c r="B120" s="13"/>
+      <c r="C120" s="13"/>
+      <c r="D120" s="13"/>
       <c r="E120" s="7" t="s">
         <v>361</v>
       </c>
-      <c r="F120" s="12"/>
-      <c r="G120" s="13"/>
+      <c r="F120" s="13"/>
+      <c r="G120" s="12"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A121" s="12" t="s">
+      <c r="A121" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="B121" s="12" t="s">
+      <c r="B121" s="13" t="s">
         <v>365</v>
       </c>
-      <c r="C121" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D121" s="12" t="s">
+      <c r="C121" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D121" s="13" t="s">
         <v>366</v>
       </c>
       <c r="E121" s="7" t="s">
         <v>360</v>
       </c>
-      <c r="F121" s="12" t="s">
+      <c r="F121" s="13" t="s">
         <v>368</v>
       </c>
-      <c r="G121" s="13" t="s">
+      <c r="G121" s="12" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A122" s="12"/>
-      <c r="B122" s="12"/>
-      <c r="C122" s="12"/>
-      <c r="D122" s="12"/>
+      <c r="A122" s="13"/>
+      <c r="B122" s="13"/>
+      <c r="C122" s="13"/>
+      <c r="D122" s="13"/>
       <c r="E122" s="9"/>
-      <c r="F122" s="12"/>
-      <c r="G122" s="13"/>
+      <c r="F122" s="13"/>
+      <c r="G122" s="12"/>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A123" s="12"/>
-      <c r="B123" s="12"/>
-      <c r="C123" s="12"/>
-      <c r="D123" s="12"/>
+      <c r="A123" s="13"/>
+      <c r="B123" s="13"/>
+      <c r="C123" s="13"/>
+      <c r="D123" s="13"/>
       <c r="E123" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="F123" s="12"/>
-      <c r="G123" s="13"/>
+      <c r="F123" s="13"/>
+      <c r="G123" s="12"/>
     </row>
     <row r="124" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A124" s="7" t="s">
@@ -4006,104 +4718,143 @@
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A127" s="12" t="s">
+      <c r="A127" s="13" t="s">
         <v>412</v>
       </c>
-      <c r="B127" s="12" t="s">
+      <c r="B127" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="C127" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D127" s="12" t="s">
+      <c r="C127" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D127" s="13" t="s">
         <v>388</v>
       </c>
       <c r="E127" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="F127" s="12" t="s">
+      <c r="F127" s="13" t="s">
         <v>391</v>
       </c>
-      <c r="G127" s="13" t="s">
+      <c r="G127" s="12" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A128" s="12"/>
-      <c r="B128" s="12"/>
-      <c r="C128" s="12"/>
-      <c r="D128" s="12"/>
+      <c r="A128" s="13"/>
+      <c r="B128" s="13"/>
+      <c r="C128" s="13"/>
+      <c r="D128" s="13"/>
       <c r="E128" s="9"/>
-      <c r="F128" s="12"/>
-      <c r="G128" s="13"/>
+      <c r="F128" s="13"/>
+      <c r="G128" s="12"/>
     </row>
     <row r="129" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A129" s="12"/>
-      <c r="B129" s="12"/>
-      <c r="C129" s="12"/>
-      <c r="D129" s="12"/>
+      <c r="A129" s="13"/>
+      <c r="B129" s="13"/>
+      <c r="C129" s="13"/>
+      <c r="D129" s="13"/>
       <c r="E129" s="7" t="s">
         <v>390</v>
       </c>
-      <c r="F129" s="12"/>
-      <c r="G129" s="13"/>
+      <c r="F129" s="13"/>
+      <c r="G129" s="12"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A130" s="12" t="s">
+      <c r="A130" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="B130" s="12" t="s">
+      <c r="B130" s="13" t="s">
         <v>394</v>
       </c>
-      <c r="C130" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D130" s="12" t="s">
+      <c r="C130" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D130" s="13" t="s">
         <v>395</v>
       </c>
       <c r="E130" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="F130" s="12" t="s">
+      <c r="F130" s="13" t="s">
         <v>398</v>
       </c>
-      <c r="G130" s="13" t="s">
+      <c r="G130" s="12" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A131" s="12"/>
-      <c r="B131" s="12"/>
-      <c r="C131" s="12"/>
-      <c r="D131" s="12"/>
+      <c r="A131" s="13"/>
+      <c r="B131" s="13"/>
+      <c r="C131" s="13"/>
+      <c r="D131" s="13"/>
       <c r="E131" s="9"/>
-      <c r="F131" s="12"/>
-      <c r="G131" s="13"/>
+      <c r="F131" s="13"/>
+      <c r="G131" s="12"/>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A132" s="12"/>
-      <c r="B132" s="12"/>
-      <c r="C132" s="12"/>
-      <c r="D132" s="12"/>
+      <c r="A132" s="13"/>
+      <c r="B132" s="13"/>
+      <c r="C132" s="13"/>
+      <c r="D132" s="13"/>
       <c r="E132" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="F132" s="12"/>
-      <c r="G132" s="13"/>
+      <c r="F132" s="13"/>
+      <c r="G132" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="G25:G31"/>
-    <mergeCell ref="A25:A31"/>
-    <mergeCell ref="B25:B31"/>
-    <mergeCell ref="C25:C31"/>
-    <mergeCell ref="D25:D31"/>
-    <mergeCell ref="F25:F31"/>
-    <mergeCell ref="A48:A56"/>
-    <mergeCell ref="B48:B56"/>
-    <mergeCell ref="C48:C56"/>
-    <mergeCell ref="D48:D56"/>
-    <mergeCell ref="G48:G56"/>
+    <mergeCell ref="G130:G132"/>
+    <mergeCell ref="A127:A129"/>
+    <mergeCell ref="B127:B129"/>
+    <mergeCell ref="C127:C129"/>
+    <mergeCell ref="D127:D129"/>
+    <mergeCell ref="F127:F129"/>
+    <mergeCell ref="G127:G129"/>
+    <mergeCell ref="A130:A132"/>
+    <mergeCell ref="B130:B132"/>
+    <mergeCell ref="C130:C132"/>
+    <mergeCell ref="D130:D132"/>
+    <mergeCell ref="F130:F132"/>
+    <mergeCell ref="G121:G123"/>
+    <mergeCell ref="A118:A120"/>
+    <mergeCell ref="B118:B120"/>
+    <mergeCell ref="C118:C120"/>
+    <mergeCell ref="D118:D120"/>
+    <mergeCell ref="F118:F120"/>
+    <mergeCell ref="G118:G120"/>
+    <mergeCell ref="A121:A123"/>
+    <mergeCell ref="B121:B123"/>
+    <mergeCell ref="C121:C123"/>
+    <mergeCell ref="D121:D123"/>
+    <mergeCell ref="F121:F123"/>
+    <mergeCell ref="G115:G117"/>
+    <mergeCell ref="A104:A110"/>
+    <mergeCell ref="B104:B110"/>
+    <mergeCell ref="C104:C110"/>
+    <mergeCell ref="D104:D110"/>
+    <mergeCell ref="F104:F110"/>
+    <mergeCell ref="G104:G110"/>
+    <mergeCell ref="A115:A117"/>
+    <mergeCell ref="B115:B117"/>
+    <mergeCell ref="C115:C117"/>
+    <mergeCell ref="D115:D117"/>
+    <mergeCell ref="F115:F117"/>
+    <mergeCell ref="D72:D78"/>
+    <mergeCell ref="F72:F78"/>
+    <mergeCell ref="G83:G85"/>
+    <mergeCell ref="A80:A82"/>
+    <mergeCell ref="B80:B82"/>
+    <mergeCell ref="C80:C82"/>
+    <mergeCell ref="D80:D82"/>
+    <mergeCell ref="F80:F82"/>
+    <mergeCell ref="G80:G82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="C83:C85"/>
+    <mergeCell ref="D83:D85"/>
+    <mergeCell ref="F83:F85"/>
     <mergeCell ref="G72:G78"/>
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A61:A67"/>
@@ -4120,56 +4871,17 @@
     <mergeCell ref="A72:A78"/>
     <mergeCell ref="B72:B78"/>
     <mergeCell ref="C72:C78"/>
-    <mergeCell ref="D72:D78"/>
-    <mergeCell ref="F72:F78"/>
-    <mergeCell ref="G83:G85"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="C80:C82"/>
-    <mergeCell ref="D80:D82"/>
-    <mergeCell ref="F80:F82"/>
-    <mergeCell ref="G80:G82"/>
-    <mergeCell ref="A83:A85"/>
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="C83:C85"/>
-    <mergeCell ref="D83:D85"/>
-    <mergeCell ref="F83:F85"/>
-    <mergeCell ref="G115:G117"/>
-    <mergeCell ref="A104:A110"/>
-    <mergeCell ref="B104:B110"/>
-    <mergeCell ref="C104:C110"/>
-    <mergeCell ref="D104:D110"/>
-    <mergeCell ref="F104:F110"/>
-    <mergeCell ref="G104:G110"/>
-    <mergeCell ref="A115:A117"/>
-    <mergeCell ref="B115:B117"/>
-    <mergeCell ref="C115:C117"/>
-    <mergeCell ref="D115:D117"/>
-    <mergeCell ref="F115:F117"/>
-    <mergeCell ref="G121:G123"/>
-    <mergeCell ref="A118:A120"/>
-    <mergeCell ref="B118:B120"/>
-    <mergeCell ref="C118:C120"/>
-    <mergeCell ref="D118:D120"/>
-    <mergeCell ref="F118:F120"/>
-    <mergeCell ref="G118:G120"/>
-    <mergeCell ref="A121:A123"/>
-    <mergeCell ref="B121:B123"/>
-    <mergeCell ref="C121:C123"/>
-    <mergeCell ref="D121:D123"/>
-    <mergeCell ref="F121:F123"/>
-    <mergeCell ref="G130:G132"/>
-    <mergeCell ref="A127:A129"/>
-    <mergeCell ref="B127:B129"/>
-    <mergeCell ref="C127:C129"/>
-    <mergeCell ref="D127:D129"/>
-    <mergeCell ref="F127:F129"/>
-    <mergeCell ref="G127:G129"/>
-    <mergeCell ref="A130:A132"/>
-    <mergeCell ref="B130:B132"/>
-    <mergeCell ref="C130:C132"/>
-    <mergeCell ref="D130:D132"/>
-    <mergeCell ref="F130:F132"/>
+    <mergeCell ref="A48:A56"/>
+    <mergeCell ref="B48:B56"/>
+    <mergeCell ref="C48:C56"/>
+    <mergeCell ref="D48:D56"/>
+    <mergeCell ref="G48:G56"/>
+    <mergeCell ref="G25:G31"/>
+    <mergeCell ref="A25:A31"/>
+    <mergeCell ref="B25:B31"/>
+    <mergeCell ref="C25:C31"/>
+    <mergeCell ref="D25:D31"/>
+    <mergeCell ref="F25:F31"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
@@ -4177,4 +4889,1284 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A839601F-91A6-426F-A380-D25008A6D01B}">
+  <dimension ref="A1:G58"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.21875" customWidth="1"/>
+    <col min="2" max="2" width="44.21875" customWidth="1"/>
+    <col min="3" max="3" width="48.88671875" customWidth="1"/>
+    <col min="4" max="4" width="59.21875" customWidth="1"/>
+    <col min="5" max="5" width="65.33203125" customWidth="1"/>
+    <col min="6" max="6" width="46.88671875" customWidth="1"/>
+    <col min="7" max="7" width="36.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+    </row>
+    <row r="2" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>592</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+    </row>
+    <row r="3" spans="1:7" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>414</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+    </row>
+    <row r="4" spans="1:7" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>416</v>
+      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+    </row>
+    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>417</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>593</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>418</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>420</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>421</v>
+      </c>
+      <c r="F9" s="18">
+        <v>2342527890</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
+        <v>594</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>424</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="18" t="s">
+        <v>595</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>428</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>430</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>432</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
+        <v>596</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>434</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>435</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="18" t="s">
+        <v>597</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>436</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>438</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="F13" s="18">
+        <v>1234567890</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="18" t="s">
+        <v>598</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>440</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>441</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="F14" s="18">
+        <v>123456789012</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="18" t="s">
+        <v>599</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>444</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>445</v>
+      </c>
+      <c r="F15" s="18">
+        <v>9999999999</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="18" t="s">
+        <v>600</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>447</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>448</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>449</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>451</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>452</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>585</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
+        <v>602</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>454</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>455</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>586</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="18" t="s">
+        <v>603</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>457</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>458</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>453</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>587</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="18" t="s">
+        <v>604</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>459</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>460</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>461</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>462</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="18" t="s">
+        <v>605</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>463</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>464</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>461</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>465</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
+        <v>606</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>466</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>467</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>468</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="18" t="s">
+        <v>607</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>469</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>470</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>471</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>588</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="18" t="s">
+        <v>608</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>472</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>473</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>590</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="18" t="s">
+        <v>609</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>475</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>476</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="G25" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="18" t="s">
+        <v>610</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>477</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>478</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>479</v>
+      </c>
+      <c r="G26" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="18" t="s">
+        <v>611</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>480</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>481</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>474</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>482</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="18" t="s">
+        <v>612</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>483</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>484</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>485</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="18" t="s">
+        <v>613</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>486</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>487</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>488</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="18" t="s">
+        <v>614</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>489</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>490</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>488</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="18" t="s">
+        <v>615</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>492</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>493</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>488</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>494</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="18" t="s">
+        <v>616</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>495</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>496</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>488</v>
+      </c>
+      <c r="F32" s="20" t="s">
+        <v>497</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="18" t="s">
+        <v>617</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>498</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>499</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>485</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="18" t="s">
+        <v>618</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>500</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>501</v>
+      </c>
+      <c r="E34" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="F34" s="18">
+        <v>9876543210</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="18" t="s">
+        <v>619</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>503</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>504</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>432</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="18" t="s">
+        <v>620</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>505</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>476</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>506</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="18" t="s">
+        <v>621</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>507</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>508</v>
+      </c>
+      <c r="E37" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="F37" s="18">
+        <v>12345</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="18" t="s">
+        <v>622</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>509</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>510</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="F38" s="18">
+        <v>123456789012</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="18" t="s">
+        <v>623</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>511</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>512</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>485</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="18" t="s">
+        <v>624</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>513</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>514</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>515</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>516</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="18" t="s">
+        <v>625</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>517</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>518</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>515</v>
+      </c>
+      <c r="F41" s="18" t="s">
+        <v>519</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="18" t="s">
+        <v>626</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>520</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>521</v>
+      </c>
+      <c r="E42" s="18" t="s">
+        <v>515</v>
+      </c>
+      <c r="F42" s="18" t="s">
+        <v>522</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="18" t="s">
+        <v>627</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>523</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>524</v>
+      </c>
+      <c r="E43" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="F43" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="18" t="s">
+        <v>628</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>526</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>527</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>528</v>
+      </c>
+      <c r="F44" s="18" t="s">
+        <v>529</v>
+      </c>
+      <c r="G44" s="18" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="18" t="s">
+        <v>629</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>531</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>532</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>528</v>
+      </c>
+      <c r="F45" s="18" t="s">
+        <v>533</v>
+      </c>
+      <c r="G45" s="18" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="18" t="s">
+        <v>630</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>534</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D46" s="18" t="s">
+        <v>535</v>
+      </c>
+      <c r="E46" s="18" t="s">
+        <v>536</v>
+      </c>
+      <c r="F46" s="18" t="s">
+        <v>537</v>
+      </c>
+      <c r="G46" s="18" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="18" t="s">
+        <v>631</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>539</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>540</v>
+      </c>
+      <c r="E47" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="F47" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="18" t="s">
+        <v>632</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>541</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>542</v>
+      </c>
+      <c r="D48" s="18" t="s">
+        <v>543</v>
+      </c>
+      <c r="E48" s="18" t="s">
+        <v>544</v>
+      </c>
+      <c r="F48" s="18" t="s">
+        <v>545</v>
+      </c>
+      <c r="G48" s="18" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="18" t="s">
+        <v>633</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>547</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>548</v>
+      </c>
+      <c r="E49" s="18" t="s">
+        <v>549</v>
+      </c>
+      <c r="F49" s="18" t="s">
+        <v>550</v>
+      </c>
+      <c r="G49" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="18" t="s">
+        <v>634</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>551</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D50" s="18" t="s">
+        <v>552</v>
+      </c>
+      <c r="E50" s="18" t="s">
+        <v>553</v>
+      </c>
+      <c r="F50" s="18" t="s">
+        <v>450</v>
+      </c>
+      <c r="G50" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="18" t="s">
+        <v>635</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>554</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>493</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>555</v>
+      </c>
+      <c r="F51" s="20" t="s">
+        <v>494</v>
+      </c>
+      <c r="G51" s="18" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>636</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>556</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="D52" s="18" t="s">
+        <v>557</v>
+      </c>
+      <c r="E52" s="18" t="s">
+        <v>558</v>
+      </c>
+      <c r="F52" s="18" t="s">
+        <v>559</v>
+      </c>
+      <c r="G52" s="18" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="18" t="s">
+        <v>637</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="C53" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D53" s="18" t="s">
+        <v>562</v>
+      </c>
+      <c r="E53" s="18" t="s">
+        <v>563</v>
+      </c>
+      <c r="F53" s="18" t="s">
+        <v>545</v>
+      </c>
+      <c r="G53" s="18" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="18" t="s">
+        <v>638</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>565</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D54" s="18" t="s">
+        <v>566</v>
+      </c>
+      <c r="E54" s="18" t="s">
+        <v>563</v>
+      </c>
+      <c r="F54" s="18" t="s">
+        <v>550</v>
+      </c>
+      <c r="G54" s="18" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="18" t="s">
+        <v>639</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>568</v>
+      </c>
+      <c r="C55" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D55" s="18" t="s">
+        <v>569</v>
+      </c>
+      <c r="E55" s="18" t="s">
+        <v>570</v>
+      </c>
+      <c r="F55" s="18" t="s">
+        <v>571</v>
+      </c>
+      <c r="G55" s="18" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="18" t="s">
+        <v>640</v>
+      </c>
+      <c r="B56" s="18" t="s">
+        <v>573</v>
+      </c>
+      <c r="C56" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D56" s="18" t="s">
+        <v>574</v>
+      </c>
+      <c r="E56" s="18" t="s">
+        <v>575</v>
+      </c>
+      <c r="F56" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" s="18" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="18" t="s">
+        <v>641</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>577</v>
+      </c>
+      <c r="C57" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D57" s="18" t="s">
+        <v>578</v>
+      </c>
+      <c r="E57" s="18" t="s">
+        <v>579</v>
+      </c>
+      <c r="F57" s="18" t="s">
+        <v>571</v>
+      </c>
+      <c r="G57" s="18" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="18" t="s">
+        <v>642</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>581</v>
+      </c>
+      <c r="C58" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="D58" s="18" t="s">
+        <v>582</v>
+      </c>
+      <c r="E58" s="18" t="s">
+        <v>575</v>
+      </c>
+      <c r="F58" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G58" s="18" t="s">
+        <v>583</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F29" r:id="rId1" xr:uid="{1912FE9C-F88C-4A80-9FFD-A8FFADB2EF2D}"/>
+    <hyperlink ref="F31" r:id="rId2" display="mailto:existing@gmail.com" xr:uid="{E69B12F3-C159-44DE-8659-E0FCDA67E7F3}"/>
+    <hyperlink ref="F32" r:id="rId3" display="mailto:new@gmail.com" xr:uid="{E87D6C8E-3901-455F-9AD9-788F5B0F0B00}"/>
+    <hyperlink ref="F51" r:id="rId4" display="mailto:existing@gmail.com" xr:uid="{8BAB50B4-4DB3-4AC7-9FC5-704B68FA0FF6}"/>
+    <hyperlink ref="F12" r:id="rId5" xr:uid="{2796E5C8-0133-4827-9CA4-FAB5FE0814A9}"/>
+    <hyperlink ref="F19" r:id="rId6" xr:uid="{5D389696-3F76-4156-BAA2-59473A00438E}"/>
+    <hyperlink ref="F25" r:id="rId7" xr:uid="{F536CD00-39C0-4BD1-B4C6-BB4E729125CD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>